<commit_message>
battery pack dummy id--date editable to admin only, always todays date and rebuild serial number from todays date(but not in reverse).
</commit_message>
<xml_diff>
--- a/models/hv/data/scan_log.xlsx
+++ b/models/hv/data/scan_log.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3036" yWindow="2340" windowWidth="11268" windowHeight="9900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="HV Dummy" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HV Dummy" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R19"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1853,6 +1853,76 @@
       <c r="Q19" s="10" t="inlineStr"/>
       <c r="R19" s="10" t="inlineStr"/>
     </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>10 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>11:48:47 AM</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>00076</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>ABA51202609101A00076</t>
+        </is>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="G20" s="15" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H20" s="17" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260076</t>
+        </is>
+      </c>
+      <c r="I20" s="17" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260077</t>
+        </is>
+      </c>
+      <c r="J20" s="17" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260078</t>
+        </is>
+      </c>
+      <c r="K20" s="17" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260079</t>
+        </is>
+      </c>
+      <c r="L20" s="15" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202609101A00076</t>
+        </is>
+      </c>
+      <c r="N20" s="18" t="inlineStr"/>
+      <c r="O20" s="18" t="inlineStr"/>
+      <c r="P20" s="18" t="inlineStr"/>
+      <c r="Q20" s="18" t="inlineStr"/>
+      <c r="R20" s="18" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
plant encoded values (either 1,2,3 or A,B,C) in Module ID , Both Accepts
</commit_message>
<xml_diff>
--- a/models/hv/data/scan_log.xlsx
+++ b/models/hv/data/scan_log.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R21"/>
+  <dimension ref="A1:R22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1989,6 +1989,76 @@
       <c r="Q21" s="10" t="inlineStr"/>
       <c r="R21" s="10" t="inlineStr"/>
     </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="15" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>21 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>3:29:39 PM</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>00001</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>ABA51202609211B00001</t>
+        </is>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H22" s="17" t="inlineStr">
+        <is>
+          <t>VX156610-E16A1109G260076</t>
+        </is>
+      </c>
+      <c r="I22" s="17" t="inlineStr">
+        <is>
+          <t>VX156610-E16A1109G260077</t>
+        </is>
+      </c>
+      <c r="J22" s="17" t="inlineStr">
+        <is>
+          <t>VX156610-E16A1109G260078</t>
+        </is>
+      </c>
+      <c r="K22" s="17" t="inlineStr">
+        <is>
+          <t>VX156610-E16A1109G260079</t>
+        </is>
+      </c>
+      <c r="L22" s="15" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M22" s="17" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202609211B00001</t>
+        </is>
+      </c>
+      <c r="N22" s="18" t="inlineStr"/>
+      <c r="O22" s="18" t="inlineStr"/>
+      <c r="P22" s="18" t="inlineStr"/>
+      <c r="Q22" s="18" t="inlineStr"/>
+      <c r="R22" s="18" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
dummy id manual gui updated, popup ask for cell_mfr and go for print
</commit_message>
<xml_diff>
--- a/models/hv/data/scan_log.xlsx
+++ b/models/hv/data/scan_log.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R30"/>
+  <dimension ref="A1:R34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2611,6 +2611,286 @@
       <c r="Q30" s="18" t="inlineStr"/>
       <c r="R30" s="18" t="inlineStr"/>
     </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>9:08:21 AM</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>00111</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00111</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t>Module Level Completed</t>
+        </is>
+      </c>
+      <c r="I31" s="9" t="inlineStr">
+        <is>
+          <t>Module Level Completed</t>
+        </is>
+      </c>
+      <c r="J31" s="9" t="inlineStr">
+        <is>
+          <t>Module Level Completed</t>
+        </is>
+      </c>
+      <c r="K31" s="9" t="inlineStr">
+        <is>
+          <t>Module Level Completed</t>
+        </is>
+      </c>
+      <c r="L31" s="7" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M31" s="9" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281A00111</t>
+        </is>
+      </c>
+      <c r="N31" s="10" t="inlineStr"/>
+      <c r="O31" s="10" t="inlineStr"/>
+      <c r="P31" s="10" t="inlineStr"/>
+      <c r="Q31" s="10" t="inlineStr"/>
+      <c r="R31" s="10" t="inlineStr"/>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="15" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="15" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="inlineStr">
+        <is>
+          <t>9:13:05 AM</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>00111</t>
+        </is>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00111</t>
+        </is>
+      </c>
+      <c r="F32" s="16" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="G32" s="15" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H32" s="17" t="inlineStr">
+        <is>
+          <t>Module Level Completed</t>
+        </is>
+      </c>
+      <c r="I32" s="17" t="inlineStr">
+        <is>
+          <t>Module Level Completed</t>
+        </is>
+      </c>
+      <c r="J32" s="17" t="inlineStr">
+        <is>
+          <t>Module Level Completed</t>
+        </is>
+      </c>
+      <c r="K32" s="17" t="inlineStr">
+        <is>
+          <t>Module Level Completed</t>
+        </is>
+      </c>
+      <c r="L32" s="15" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M32" s="17" t="inlineStr">
+        <is>
+          <t>VQ150020:ABA51202605281A00111</t>
+        </is>
+      </c>
+      <c r="N32" s="18" t="inlineStr"/>
+      <c r="O32" s="18" t="inlineStr"/>
+      <c r="P32" s="18" t="inlineStr"/>
+      <c r="Q32" s="18" t="inlineStr"/>
+      <c r="R32" s="18" t="inlineStr"/>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="7" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>09 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>9:17:37 AM</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>00111</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>ABA51202610091A00111</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H33" s="9" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260076</t>
+        </is>
+      </c>
+      <c r="I33" s="9" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260077</t>
+        </is>
+      </c>
+      <c r="J33" s="9" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260078</t>
+        </is>
+      </c>
+      <c r="K33" s="9" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260079</t>
+        </is>
+      </c>
+      <c r="L33" s="7" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M33" s="9" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202610091A00111</t>
+        </is>
+      </c>
+      <c r="N33" s="10" t="inlineStr"/>
+      <c r="O33" s="10" t="inlineStr"/>
+      <c r="P33" s="10" t="inlineStr"/>
+      <c r="Q33" s="10" t="inlineStr"/>
+      <c r="R33" s="10" t="inlineStr"/>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="15" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>09 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="inlineStr">
+        <is>
+          <t>9:22:00 AM</t>
+        </is>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>00112</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>ABA51202610091A00112</t>
+        </is>
+      </c>
+      <c r="F34" s="16" t="inlineStr">
+        <is>
+          <t>112</t>
+        </is>
+      </c>
+      <c r="G34" s="15" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H34" s="17" t="inlineStr">
+        <is>
+          <t>VQ150060-E1311109G260076</t>
+        </is>
+      </c>
+      <c r="I34" s="17" t="inlineStr">
+        <is>
+          <t>VQ150060-E1311109G260077</t>
+        </is>
+      </c>
+      <c r="J34" s="17" t="inlineStr">
+        <is>
+          <t>VQ150060-E1311109G260078</t>
+        </is>
+      </c>
+      <c r="K34" s="17" t="inlineStr">
+        <is>
+          <t>VQ150060-E1311109G260079</t>
+        </is>
+      </c>
+      <c r="L34" s="15" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M34" s="17" t="inlineStr">
+        <is>
+          <t>VQ150020:ABA51202610091A00112</t>
+        </is>
+      </c>
+      <c r="N34" s="18" t="inlineStr"/>
+      <c r="O34" s="18" t="inlineStr"/>
+      <c r="P34" s="18" t="inlineStr"/>
+      <c r="Q34" s="18" t="inlineStr"/>
+      <c r="R34" s="18" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
users.json and pack_session.json files are replaced by respective .db files
</commit_message>
<xml_diff>
--- a/models/hv/data/scan_log.xlsx
+++ b/models/hv/data/scan_log.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R52"/>
+  <dimension ref="A1:R56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4091,6 +4091,270 @@
       <c r="Q52" s="18" t="inlineStr"/>
       <c r="R52" s="18" t="inlineStr"/>
     </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="7" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>13 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>9:21:33 AM</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>00111</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>ABA51202610131R00111</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="inlineStr"/>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H53" s="9" t="inlineStr">
+        <is>
+          <t>VQ150060-E1311109G260076</t>
+        </is>
+      </c>
+      <c r="I53" s="9" t="inlineStr">
+        <is>
+          <t>VQ150060-E1311109G260077</t>
+        </is>
+      </c>
+      <c r="J53" s="9" t="inlineStr">
+        <is>
+          <t>VQ150060-E1311109G260078</t>
+        </is>
+      </c>
+      <c r="K53" s="9" t="inlineStr">
+        <is>
+          <t>VQ150060-E1311109G260079</t>
+        </is>
+      </c>
+      <c r="L53" s="7" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M53" s="9" t="inlineStr">
+        <is>
+          <t>VQ150020:ABA51202610131R00111</t>
+        </is>
+      </c>
+      <c r="N53" s="10" t="inlineStr"/>
+      <c r="O53" s="10" t="inlineStr"/>
+      <c r="P53" s="10" t="inlineStr"/>
+      <c r="Q53" s="10" t="inlineStr"/>
+      <c r="R53" s="10" t="inlineStr"/>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="15" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="15" t="inlineStr">
+        <is>
+          <t>13 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C54" s="15" t="inlineStr">
+        <is>
+          <t>9:50:11 AM</t>
+        </is>
+      </c>
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>00011</t>
+        </is>
+      </c>
+      <c r="E54" s="17" t="inlineStr">
+        <is>
+          <t>ABA51202610131U00011</t>
+        </is>
+      </c>
+      <c r="F54" s="16" t="inlineStr"/>
+      <c r="G54" s="15" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H54" s="17" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260076</t>
+        </is>
+      </c>
+      <c r="I54" s="17" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260077</t>
+        </is>
+      </c>
+      <c r="J54" s="17" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260078</t>
+        </is>
+      </c>
+      <c r="K54" s="17" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260079</t>
+        </is>
+      </c>
+      <c r="L54" s="15" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M54" s="17" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202610131U00011</t>
+        </is>
+      </c>
+      <c r="N54" s="18" t="inlineStr"/>
+      <c r="O54" s="18" t="inlineStr"/>
+      <c r="P54" s="18" t="inlineStr"/>
+      <c r="Q54" s="18" t="inlineStr"/>
+      <c r="R54" s="18" t="inlineStr"/>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="7" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>13 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>10:10:56 AM</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>00012</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>ABA51202610131R00012</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="inlineStr"/>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H55" s="9" t="inlineStr">
+        <is>
+          <t>VQ150060-E1311109G260076</t>
+        </is>
+      </c>
+      <c r="I55" s="9" t="inlineStr">
+        <is>
+          <t>VQ150060-E1311109G260077</t>
+        </is>
+      </c>
+      <c r="J55" s="9" t="inlineStr">
+        <is>
+          <t>VQ150060-E1311109G260078</t>
+        </is>
+      </c>
+      <c r="K55" s="9" t="inlineStr">
+        <is>
+          <t>VQ150060-E1311109G260079</t>
+        </is>
+      </c>
+      <c r="L55" s="7" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M55" s="9" t="inlineStr">
+        <is>
+          <t>VQ150020:ABA51202610131R00012</t>
+        </is>
+      </c>
+      <c r="N55" s="10" t="inlineStr"/>
+      <c r="O55" s="10" t="inlineStr"/>
+      <c r="P55" s="10" t="inlineStr"/>
+      <c r="Q55" s="10" t="inlineStr"/>
+      <c r="R55" s="10" t="inlineStr"/>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="15" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="15" t="inlineStr">
+        <is>
+          <t>13 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C56" s="15" t="inlineStr">
+        <is>
+          <t>10:25:32 AM</t>
+        </is>
+      </c>
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>00013</t>
+        </is>
+      </c>
+      <c r="E56" s="17" t="inlineStr">
+        <is>
+          <t>ABA51202610131R00013</t>
+        </is>
+      </c>
+      <c r="F56" s="16" t="inlineStr"/>
+      <c r="G56" s="15" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H56" s="17" t="inlineStr">
+        <is>
+          <t>VQ150060-E1311109G260076</t>
+        </is>
+      </c>
+      <c r="I56" s="17" t="inlineStr">
+        <is>
+          <t>VQ150060-E1311109G260077</t>
+        </is>
+      </c>
+      <c r="J56" s="17" t="inlineStr">
+        <is>
+          <t>VQ150060-E1311109G260078</t>
+        </is>
+      </c>
+      <c r="K56" s="17" t="inlineStr">
+        <is>
+          <t>VQ150060-E1311109G260071</t>
+        </is>
+      </c>
+      <c r="L56" s="15" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M56" s="17" t="inlineStr">
+        <is>
+          <t>VQ150020:ABA51202610131R00013</t>
+        </is>
+      </c>
+      <c r="N56" s="18" t="inlineStr"/>
+      <c r="O56" s="18" t="inlineStr"/>
+      <c r="P56" s="18" t="inlineStr"/>
+      <c r="Q56" s="18" t="inlineStr"/>
+      <c r="R56" s="18" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
unused code removed, format corrected, explained some function in comment lines
</commit_message>
<xml_diff>
--- a/models/hv/data/scan_log.xlsx
+++ b/models/hv/data/scan_log.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R56"/>
+  <dimension ref="A1:R57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4355,6 +4355,72 @@
       <c r="Q56" s="18" t="inlineStr"/>
       <c r="R56" s="18" t="inlineStr"/>
     </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="7" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>14 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>10:22:41 AM</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>00014</t>
+        </is>
+      </c>
+      <c r="E57" s="9" t="inlineStr">
+        <is>
+          <t>ABA51202610141U00014</t>
+        </is>
+      </c>
+      <c r="F57" s="8" t="inlineStr"/>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H57" s="9" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260076</t>
+        </is>
+      </c>
+      <c r="I57" s="9" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260077</t>
+        </is>
+      </c>
+      <c r="J57" s="9" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260078</t>
+        </is>
+      </c>
+      <c r="K57" s="9" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260071</t>
+        </is>
+      </c>
+      <c r="L57" s="7" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M57" s="9" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202610141U00014</t>
+        </is>
+      </c>
+      <c r="N57" s="10" t="inlineStr"/>
+      <c r="O57" s="10" t="inlineStr"/>
+      <c r="P57" s="10" t="inlineStr"/>
+      <c r="Q57" s="10" t="inlineStr"/>
+      <c r="R57" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
removed unnecessary code-- v2.0
</commit_message>
<xml_diff>
--- a/models/hv/data/scan_log.xlsx
+++ b/models/hv/data/scan_log.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R59"/>
+  <dimension ref="A1:R61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4553,6 +4553,138 @@
       <c r="Q59" s="10" t="inlineStr"/>
       <c r="R59" s="10" t="inlineStr"/>
     </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="15" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="15" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C60" s="15" t="inlineStr">
+        <is>
+          <t>3:11:04 PM</t>
+        </is>
+      </c>
+      <c r="D60" s="16" t="inlineStr">
+        <is>
+          <t>00111</t>
+        </is>
+      </c>
+      <c r="E60" s="17" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00111</t>
+        </is>
+      </c>
+      <c r="F60" s="16" t="inlineStr"/>
+      <c r="G60" s="15" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H60" s="17" t="inlineStr">
+        <is>
+          <t>Module Level Completed</t>
+        </is>
+      </c>
+      <c r="I60" s="17" t="inlineStr">
+        <is>
+          <t>Module Level Completed</t>
+        </is>
+      </c>
+      <c r="J60" s="17" t="inlineStr">
+        <is>
+          <t>Module Level Completed</t>
+        </is>
+      </c>
+      <c r="K60" s="17" t="inlineStr">
+        <is>
+          <t>Module Level Completed</t>
+        </is>
+      </c>
+      <c r="L60" s="15" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M60" s="17" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00111</t>
+        </is>
+      </c>
+      <c r="N60" s="18" t="inlineStr"/>
+      <c r="O60" s="18" t="inlineStr"/>
+      <c r="P60" s="18" t="inlineStr"/>
+      <c r="Q60" s="18" t="inlineStr"/>
+      <c r="R60" s="18" t="inlineStr"/>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>3:13:04 PM</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>00111</t>
+        </is>
+      </c>
+      <c r="E61" s="9" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00111</t>
+        </is>
+      </c>
+      <c r="F61" s="8" t="inlineStr"/>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H61" s="9" t="inlineStr">
+        <is>
+          <t>Module Level Completed</t>
+        </is>
+      </c>
+      <c r="I61" s="9" t="inlineStr">
+        <is>
+          <t>Module Level Completed</t>
+        </is>
+      </c>
+      <c r="J61" s="9" t="inlineStr">
+        <is>
+          <t>Module Level Completed</t>
+        </is>
+      </c>
+      <c r="K61" s="9" t="inlineStr">
+        <is>
+          <t>Module Level Completed</t>
+        </is>
+      </c>
+      <c r="L61" s="7" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M61" s="9" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00111</t>
+        </is>
+      </c>
+      <c r="N61" s="10" t="inlineStr"/>
+      <c r="O61" s="10" t="inlineStr"/>
+      <c r="P61" s="10" t="inlineStr"/>
+      <c r="Q61" s="10" t="inlineStr"/>
+      <c r="R61" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
saved label for api set in admin settings
</commit_message>
<xml_diff>
--- a/models/hv/data/scan_log.xlsx
+++ b/models/hv/data/scan_log.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T115"/>
+  <dimension ref="A1:T120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8786,6 +8786,358 @@
         </is>
       </c>
     </row>
+    <row r="116" ht="18" customHeight="1">
+      <c r="A116" s="19" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="19" t="inlineStr">
+        <is>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C116" s="19" t="inlineStr">
+        <is>
+          <t>12:27:14 PM</t>
+        </is>
+      </c>
+      <c r="D116" s="20" t="inlineStr">
+        <is>
+          <t>99999</t>
+        </is>
+      </c>
+      <c r="E116" s="21" t="inlineStr">
+        <is>
+          <t>ABA51202610261U99999</t>
+        </is>
+      </c>
+      <c r="F116" s="20" t="inlineStr">
+        <is>
+          <t>99999</t>
+        </is>
+      </c>
+      <c r="G116" s="19" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H116" s="21" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260076</t>
+        </is>
+      </c>
+      <c r="I116" s="21" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260075</t>
+        </is>
+      </c>
+      <c r="J116" s="21" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260074</t>
+        </is>
+      </c>
+      <c r="K116" s="21" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260073</t>
+        </is>
+      </c>
+      <c r="L116" s="19" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M116" s="21" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202610261U99999</t>
+        </is>
+      </c>
+      <c r="N116" s="22" t="inlineStr"/>
+      <c r="O116" s="22" t="inlineStr"/>
+      <c r="P116" s="22" t="inlineStr"/>
+      <c r="Q116" s="22" t="inlineStr"/>
+      <c r="R116" s="22" t="inlineStr"/>
+      <c r="S116" s="19" t="inlineStr"/>
+      <c r="T116" s="19" t="inlineStr"/>
+    </row>
+    <row r="117" ht="18" customHeight="1">
+      <c r="A117" s="1" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="1" t="inlineStr">
+        <is>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C117" s="1" t="inlineStr">
+        <is>
+          <t>12:28:44 PM</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>00001</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>ABA51202610261U00001</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr"/>
+      <c r="G117" s="1" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H117" s="3" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260076</t>
+        </is>
+      </c>
+      <c r="I117" s="3" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260074</t>
+        </is>
+      </c>
+      <c r="J117" s="3" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260073</t>
+        </is>
+      </c>
+      <c r="K117" s="3" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260072</t>
+        </is>
+      </c>
+      <c r="L117" s="1" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M117" s="3" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202610261U00001</t>
+        </is>
+      </c>
+      <c r="N117" s="4" t="inlineStr"/>
+      <c r="O117" s="4" t="inlineStr"/>
+      <c r="P117" s="4" t="inlineStr"/>
+      <c r="Q117" s="4" t="inlineStr"/>
+      <c r="R117" s="4" t="inlineStr"/>
+      <c r="S117" s="1" t="inlineStr"/>
+      <c r="T117" s="1" t="inlineStr"/>
+    </row>
+    <row r="118" ht="18" customHeight="1">
+      <c r="A118" s="19" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="19" t="inlineStr">
+        <is>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C118" s="19" t="inlineStr">
+        <is>
+          <t>12:29:07 PM</t>
+        </is>
+      </c>
+      <c r="D118" s="20" t="inlineStr">
+        <is>
+          <t>99999</t>
+        </is>
+      </c>
+      <c r="E118" s="21" t="inlineStr">
+        <is>
+          <t>ABA51202610261U99999</t>
+        </is>
+      </c>
+      <c r="F118" s="20" t="inlineStr"/>
+      <c r="G118" s="19" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H118" s="21" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260076</t>
+        </is>
+      </c>
+      <c r="I118" s="21" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260077</t>
+        </is>
+      </c>
+      <c r="J118" s="21" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260079</t>
+        </is>
+      </c>
+      <c r="K118" s="21" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260078</t>
+        </is>
+      </c>
+      <c r="L118" s="19" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M118" s="21" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202610261U99999</t>
+        </is>
+      </c>
+      <c r="N118" s="22" t="inlineStr"/>
+      <c r="O118" s="22" t="inlineStr"/>
+      <c r="P118" s="22" t="inlineStr"/>
+      <c r="Q118" s="22" t="inlineStr"/>
+      <c r="R118" s="22" t="inlineStr"/>
+      <c r="S118" s="19" t="inlineStr"/>
+      <c r="T118" s="19" t="inlineStr"/>
+    </row>
+    <row r="119" ht="18" customHeight="1">
+      <c r="A119" s="1" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="1" t="inlineStr">
+        <is>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C119" s="1" t="inlineStr">
+        <is>
+          <t>12:34:07 PM</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>99999</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>ABA51202610261U99999</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G119" s="1" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H119" s="3" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260076</t>
+        </is>
+      </c>
+      <c r="I119" s="3" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260074</t>
+        </is>
+      </c>
+      <c r="J119" s="3" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260072</t>
+        </is>
+      </c>
+      <c r="K119" s="3" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260070</t>
+        </is>
+      </c>
+      <c r="L119" s="1" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M119" s="3" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202610261U99999</t>
+        </is>
+      </c>
+      <c r="N119" s="4" t="inlineStr"/>
+      <c r="O119" s="4" t="inlineStr"/>
+      <c r="P119" s="4" t="inlineStr"/>
+      <c r="Q119" s="4" t="inlineStr"/>
+      <c r="R119" s="4" t="inlineStr"/>
+      <c r="S119" s="1" t="inlineStr"/>
+      <c r="T119" s="1" t="inlineStr"/>
+    </row>
+    <row r="120" ht="18" customHeight="1">
+      <c r="A120" s="19" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="19" t="inlineStr">
+        <is>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C120" s="19" t="inlineStr">
+        <is>
+          <t>12:34:42 PM</t>
+        </is>
+      </c>
+      <c r="D120" s="20" t="inlineStr">
+        <is>
+          <t>A0000</t>
+        </is>
+      </c>
+      <c r="E120" s="21" t="inlineStr">
+        <is>
+          <t>ABA51202610261UA0000</t>
+        </is>
+      </c>
+      <c r="F120" s="20" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G120" s="19" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H120" s="21" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260076</t>
+        </is>
+      </c>
+      <c r="I120" s="21" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260075</t>
+        </is>
+      </c>
+      <c r="J120" s="21" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260077</t>
+        </is>
+      </c>
+      <c r="K120" s="21" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260078</t>
+        </is>
+      </c>
+      <c r="L120" s="19" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M120" s="21" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202610261UA0000</t>
+        </is>
+      </c>
+      <c r="N120" s="22" t="inlineStr"/>
+      <c r="O120" s="22" t="inlineStr"/>
+      <c r="P120" s="22" t="inlineStr"/>
+      <c r="Q120" s="22" t="inlineStr"/>
+      <c r="R120" s="22" t="inlineStr"/>
+      <c r="S120" s="19" t="inlineStr"/>
+      <c r="T120" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
hv sw ts with gui backend logic for module var label and other minor code updated
</commit_message>
<xml_diff>
--- a/models/hv/data/scan_log.xlsx
+++ b/models/hv/data/scan_log.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T139"/>
+  <dimension ref="A1:T150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -10446,6 +10446,650 @@
       <c r="S139" s="1" t="inlineStr"/>
       <c r="T139" s="1" t="inlineStr"/>
     </row>
+    <row r="140" ht="18" customHeight="1">
+      <c r="A140" s="19" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" s="19" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C140" s="19" t="inlineStr">
+        <is>
+          <t>06:46:18 PM</t>
+        </is>
+      </c>
+      <c r="D140" s="20" t="inlineStr">
+        <is>
+          <t>00011</t>
+        </is>
+      </c>
+      <c r="E140" s="21" t="inlineStr">
+        <is>
+          <t>ACS21202610291R00011</t>
+        </is>
+      </c>
+      <c r="F140" s="20" t="inlineStr"/>
+      <c r="G140" s="19" t="inlineStr">
+        <is>
+          <t>SW_RH_8P</t>
+        </is>
+      </c>
+      <c r="H140" s="21" t="inlineStr">
+        <is>
+          <t>BP00000141-H1311130J260001</t>
+        </is>
+      </c>
+      <c r="I140" s="21" t="inlineStr">
+        <is>
+          <t>BP00000141-H1311130J260002</t>
+        </is>
+      </c>
+      <c r="J140" s="21" t="inlineStr">
+        <is>
+          <t>BP00000141-H1311130J260003</t>
+        </is>
+      </c>
+      <c r="K140" s="21" t="inlineStr">
+        <is>
+          <t>BP00000141-H1311130J260004</t>
+        </is>
+      </c>
+      <c r="L140" s="19" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M140" s="21" t="inlineStr">
+        <is>
+          <t>BP00000129:ACS21202610291R00011</t>
+        </is>
+      </c>
+      <c r="N140" s="22" t="inlineStr"/>
+      <c r="O140" s="22" t="inlineStr"/>
+      <c r="P140" s="22" t="inlineStr"/>
+      <c r="Q140" s="22" t="inlineStr"/>
+      <c r="R140" s="22" t="inlineStr"/>
+      <c r="S140" s="19" t="inlineStr"/>
+      <c r="T140" s="19" t="inlineStr"/>
+    </row>
+    <row r="141" ht="18" customHeight="1">
+      <c r="A141" s="1" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="1" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C141" s="1" t="inlineStr">
+        <is>
+          <t>07:29:26 PM</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>00011</t>
+        </is>
+      </c>
+      <c r="E141" s="3" t="inlineStr">
+        <is>
+          <t>ACS11202610291R00011</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr"/>
+      <c r="G141" s="1" t="inlineStr">
+        <is>
+          <t>SW_LH_8P</t>
+        </is>
+      </c>
+      <c r="H141" s="3" t="inlineStr">
+        <is>
+          <t>BP00000140-G1311129J260001</t>
+        </is>
+      </c>
+      <c r="I141" s="3" t="inlineStr">
+        <is>
+          <t>BP00000141-H1311129J260002</t>
+        </is>
+      </c>
+      <c r="J141" s="3" t="inlineStr"/>
+      <c r="K141" s="3" t="inlineStr"/>
+      <c r="L141" s="1" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M141" s="3" t="inlineStr">
+        <is>
+          <t>BP00000129:ACS11202610291R00011</t>
+        </is>
+      </c>
+      <c r="N141" s="4" t="inlineStr"/>
+      <c r="O141" s="4" t="inlineStr"/>
+      <c r="P141" s="4" t="inlineStr"/>
+      <c r="Q141" s="4" t="inlineStr"/>
+      <c r="R141" s="4" t="inlineStr"/>
+      <c r="S141" s="1" t="inlineStr"/>
+      <c r="T141" s="1" t="inlineStr"/>
+    </row>
+    <row r="142" ht="18" customHeight="1">
+      <c r="A142" s="19" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="19" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C142" s="19" t="inlineStr">
+        <is>
+          <t>07:31:23 PM</t>
+        </is>
+      </c>
+      <c r="D142" s="20" t="inlineStr">
+        <is>
+          <t>00011</t>
+        </is>
+      </c>
+      <c r="E142" s="21" t="inlineStr">
+        <is>
+          <t>ADT11202610291R00011</t>
+        </is>
+      </c>
+      <c r="F142" s="20" t="inlineStr"/>
+      <c r="G142" s="19" t="inlineStr">
+        <is>
+          <t>TS_8P</t>
+        </is>
+      </c>
+      <c r="H142" s="21" t="inlineStr">
+        <is>
+          <t>BP00000131-M1311130J260006</t>
+        </is>
+      </c>
+      <c r="I142" s="21" t="inlineStr"/>
+      <c r="J142" s="21" t="inlineStr"/>
+      <c r="K142" s="21" t="inlineStr"/>
+      <c r="L142" s="19" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M142" s="21" t="inlineStr">
+        <is>
+          <t>BP00000131:ADT11202610291R00011</t>
+        </is>
+      </c>
+      <c r="N142" s="22" t="inlineStr"/>
+      <c r="O142" s="22" t="inlineStr"/>
+      <c r="P142" s="22" t="inlineStr"/>
+      <c r="Q142" s="22" t="inlineStr"/>
+      <c r="R142" s="22" t="inlineStr"/>
+      <c r="S142" s="19" t="inlineStr"/>
+      <c r="T142" s="19" t="inlineStr"/>
+    </row>
+    <row r="143" ht="18" customHeight="1">
+      <c r="A143" s="1" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="1" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C143" s="1" t="inlineStr">
+        <is>
+          <t>07:32:59 PM</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>00011</t>
+        </is>
+      </c>
+      <c r="E143" s="3" t="inlineStr">
+        <is>
+          <t>ACS51202610291R00011</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr"/>
+      <c r="G143" s="1" t="inlineStr">
+        <is>
+          <t>SW_LH_10P_6</t>
+        </is>
+      </c>
+      <c r="H143" s="3" t="inlineStr">
+        <is>
+          <t>BP00000147-L1311130J260005</t>
+        </is>
+      </c>
+      <c r="I143" s="3" t="inlineStr">
+        <is>
+          <t>BP00000148-K1311130J260004</t>
+        </is>
+      </c>
+      <c r="J143" s="3" t="inlineStr"/>
+      <c r="K143" s="3" t="inlineStr"/>
+      <c r="L143" s="1" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M143" s="3" t="inlineStr">
+        <is>
+          <t>BP00000130:ACS51202610291R00011</t>
+        </is>
+      </c>
+      <c r="N143" s="4" t="inlineStr"/>
+      <c r="O143" s="4" t="inlineStr"/>
+      <c r="P143" s="4" t="inlineStr"/>
+      <c r="Q143" s="4" t="inlineStr"/>
+      <c r="R143" s="4" t="inlineStr"/>
+      <c r="S143" s="1" t="inlineStr"/>
+      <c r="T143" s="1" t="inlineStr"/>
+    </row>
+    <row r="144" ht="18" customHeight="1">
+      <c r="A144" s="19" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="19" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C144" s="19" t="inlineStr">
+        <is>
+          <t>07:36:26 PM</t>
+        </is>
+      </c>
+      <c r="D144" s="20" t="inlineStr">
+        <is>
+          <t>00011</t>
+        </is>
+      </c>
+      <c r="E144" s="21" t="inlineStr">
+        <is>
+          <t>ACS51202610291R00011</t>
+        </is>
+      </c>
+      <c r="F144" s="20" t="inlineStr"/>
+      <c r="G144" s="19" t="inlineStr">
+        <is>
+          <t>SW_LH_10P_6</t>
+        </is>
+      </c>
+      <c r="H144" s="21" t="inlineStr">
+        <is>
+          <t>BP00000148-K1311130J260004</t>
+        </is>
+      </c>
+      <c r="I144" s="21" t="inlineStr">
+        <is>
+          <t>BP00000147-L1311130J260005</t>
+        </is>
+      </c>
+      <c r="J144" s="21" t="inlineStr"/>
+      <c r="K144" s="21" t="inlineStr"/>
+      <c r="L144" s="19" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M144" s="21" t="inlineStr">
+        <is>
+          <t>BP00000130:ACS51202610291R00011</t>
+        </is>
+      </c>
+      <c r="N144" s="22" t="inlineStr"/>
+      <c r="O144" s="22" t="inlineStr"/>
+      <c r="P144" s="22" t="inlineStr"/>
+      <c r="Q144" s="22" t="inlineStr"/>
+      <c r="R144" s="22" t="inlineStr"/>
+      <c r="S144" s="19" t="inlineStr"/>
+      <c r="T144" s="19" t="inlineStr"/>
+    </row>
+    <row r="145" ht="18" customHeight="1">
+      <c r="A145" s="1" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" s="1" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C145" s="1" t="inlineStr">
+        <is>
+          <t>07:36:49 PM</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>00011</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="inlineStr">
+        <is>
+          <t>ACS51202610291R00011</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr"/>
+      <c r="G145" s="1" t="inlineStr">
+        <is>
+          <t>SW_LH_10P_6</t>
+        </is>
+      </c>
+      <c r="H145" s="3" t="inlineStr">
+        <is>
+          <t>BP00000147-L1311130J260005</t>
+        </is>
+      </c>
+      <c r="I145" s="3" t="inlineStr">
+        <is>
+          <t>BP00000148-K1311130J260004</t>
+        </is>
+      </c>
+      <c r="J145" s="3" t="inlineStr"/>
+      <c r="K145" s="3" t="inlineStr"/>
+      <c r="L145" s="1" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M145" s="3" t="inlineStr">
+        <is>
+          <t>BP00000130:ACS51202610291R00011</t>
+        </is>
+      </c>
+      <c r="N145" s="4" t="inlineStr"/>
+      <c r="O145" s="4" t="inlineStr"/>
+      <c r="P145" s="4" t="inlineStr"/>
+      <c r="Q145" s="4" t="inlineStr"/>
+      <c r="R145" s="4" t="inlineStr"/>
+      <c r="S145" s="1" t="inlineStr"/>
+      <c r="T145" s="1" t="inlineStr"/>
+    </row>
+    <row r="146" ht="18" customHeight="1">
+      <c r="A146" s="19" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="19" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C146" s="19" t="inlineStr">
+        <is>
+          <t>07:37:49 PM</t>
+        </is>
+      </c>
+      <c r="D146" s="20" t="inlineStr">
+        <is>
+          <t>00012</t>
+        </is>
+      </c>
+      <c r="E146" s="21" t="inlineStr">
+        <is>
+          <t>ADT31202610291R00012</t>
+        </is>
+      </c>
+      <c r="F146" s="20" t="inlineStr"/>
+      <c r="G146" s="19" t="inlineStr">
+        <is>
+          <t>TS_10P_6</t>
+        </is>
+      </c>
+      <c r="H146" s="21" t="inlineStr">
+        <is>
+          <t>BP00000132-O1311130J260008</t>
+        </is>
+      </c>
+      <c r="I146" s="21" t="inlineStr"/>
+      <c r="J146" s="21" t="inlineStr"/>
+      <c r="K146" s="21" t="inlineStr"/>
+      <c r="L146" s="19" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M146" s="21" t="inlineStr">
+        <is>
+          <t>BP00000132:ADT31202610291R00012</t>
+        </is>
+      </c>
+      <c r="N146" s="22" t="inlineStr"/>
+      <c r="O146" s="22" t="inlineStr"/>
+      <c r="P146" s="22" t="inlineStr"/>
+      <c r="Q146" s="22" t="inlineStr"/>
+      <c r="R146" s="22" t="inlineStr"/>
+      <c r="S146" s="19" t="inlineStr"/>
+      <c r="T146" s="19" t="inlineStr"/>
+    </row>
+    <row r="147" ht="18" customHeight="1">
+      <c r="A147" s="1" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="1" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C147" s="1" t="inlineStr">
+        <is>
+          <t>07:38:12 PM</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>00012</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>ADT31202610291R00012</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr"/>
+      <c r="G147" s="1" t="inlineStr">
+        <is>
+          <t>TS_10P_6</t>
+        </is>
+      </c>
+      <c r="H147" s="3" t="inlineStr">
+        <is>
+          <t>BP00000132-O1311130J260008</t>
+        </is>
+      </c>
+      <c r="I147" s="3" t="inlineStr"/>
+      <c r="J147" s="3" t="inlineStr"/>
+      <c r="K147" s="3" t="inlineStr"/>
+      <c r="L147" s="1" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M147" s="3" t="inlineStr">
+        <is>
+          <t>BP00000132:ADT31202610291R00012</t>
+        </is>
+      </c>
+      <c r="N147" s="4" t="inlineStr"/>
+      <c r="O147" s="4" t="inlineStr"/>
+      <c r="P147" s="4" t="inlineStr"/>
+      <c r="Q147" s="4" t="inlineStr"/>
+      <c r="R147" s="4" t="inlineStr"/>
+      <c r="S147" s="1" t="inlineStr"/>
+      <c r="T147" s="1" t="inlineStr"/>
+    </row>
+    <row r="148" ht="18" customHeight="1">
+      <c r="A148" s="19" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" s="19" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C148" s="19" t="inlineStr">
+        <is>
+          <t>07:38:23 PM</t>
+        </is>
+      </c>
+      <c r="D148" s="20" t="inlineStr">
+        <is>
+          <t>00012</t>
+        </is>
+      </c>
+      <c r="E148" s="21" t="inlineStr">
+        <is>
+          <t>ADT31202610291R00012</t>
+        </is>
+      </c>
+      <c r="F148" s="20" t="inlineStr"/>
+      <c r="G148" s="19" t="inlineStr">
+        <is>
+          <t>TS_10P_6</t>
+        </is>
+      </c>
+      <c r="H148" s="21" t="inlineStr">
+        <is>
+          <t>BP00000132-O1311130J260009</t>
+        </is>
+      </c>
+      <c r="I148" s="21" t="inlineStr"/>
+      <c r="J148" s="21" t="inlineStr"/>
+      <c r="K148" s="21" t="inlineStr"/>
+      <c r="L148" s="19" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M148" s="21" t="inlineStr">
+        <is>
+          <t>BP00000132:ADT31202610291R00012</t>
+        </is>
+      </c>
+      <c r="N148" s="22" t="inlineStr"/>
+      <c r="O148" s="22" t="inlineStr"/>
+      <c r="P148" s="22" t="inlineStr"/>
+      <c r="Q148" s="22" t="inlineStr"/>
+      <c r="R148" s="22" t="inlineStr"/>
+      <c r="S148" s="19" t="inlineStr"/>
+      <c r="T148" s="19" t="inlineStr"/>
+    </row>
+    <row r="149" ht="18" customHeight="1">
+      <c r="A149" s="1" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" s="1" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C149" s="1" t="inlineStr">
+        <is>
+          <t>07:41:53 PM</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>00012</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>ADT31202610291R00012</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr"/>
+      <c r="G149" s="1" t="inlineStr">
+        <is>
+          <t>TS_10P_6</t>
+        </is>
+      </c>
+      <c r="H149" s="3" t="inlineStr">
+        <is>
+          <t>BP00000132-O1311130J260008</t>
+        </is>
+      </c>
+      <c r="I149" s="3" t="inlineStr"/>
+      <c r="J149" s="3" t="inlineStr"/>
+      <c r="K149" s="3" t="inlineStr"/>
+      <c r="L149" s="1" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M149" s="3" t="inlineStr">
+        <is>
+          <t>BP00000132:ADT31202610291R00012</t>
+        </is>
+      </c>
+      <c r="N149" s="4" t="inlineStr"/>
+      <c r="O149" s="4" t="inlineStr"/>
+      <c r="P149" s="4" t="inlineStr"/>
+      <c r="Q149" s="4" t="inlineStr"/>
+      <c r="R149" s="4" t="inlineStr"/>
+      <c r="S149" s="1" t="inlineStr"/>
+      <c r="T149" s="1" t="inlineStr"/>
+    </row>
+    <row r="150" ht="18" customHeight="1">
+      <c r="A150" s="19" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" s="19" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C150" s="19" t="inlineStr">
+        <is>
+          <t>07:42:03 PM</t>
+        </is>
+      </c>
+      <c r="D150" s="20" t="inlineStr">
+        <is>
+          <t>00013</t>
+        </is>
+      </c>
+      <c r="E150" s="21" t="inlineStr">
+        <is>
+          <t>ADT31202610291R00013</t>
+        </is>
+      </c>
+      <c r="F150" s="20" t="inlineStr"/>
+      <c r="G150" s="19" t="inlineStr">
+        <is>
+          <t>TS_10P_6</t>
+        </is>
+      </c>
+      <c r="H150" s="21" t="inlineStr">
+        <is>
+          <t>BP00000132-O1311130J260008</t>
+        </is>
+      </c>
+      <c r="I150" s="21" t="inlineStr"/>
+      <c r="J150" s="21" t="inlineStr"/>
+      <c r="K150" s="21" t="inlineStr"/>
+      <c r="L150" s="19" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M150" s="21" t="inlineStr">
+        <is>
+          <t>BP00000132:ADT31202610291R00013</t>
+        </is>
+      </c>
+      <c r="N150" s="22" t="inlineStr"/>
+      <c r="O150" s="22" t="inlineStr"/>
+      <c r="P150" s="22" t="inlineStr"/>
+      <c r="Q150" s="22" t="inlineStr"/>
+      <c r="R150" s="22" t="inlineStr"/>
+      <c r="S150" s="19" t="inlineStr"/>
+      <c r="T150" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>